<commit_message>
added fuse holder to spreadsheet
</commit_message>
<xml_diff>
--- a/astromech/Electrical/Power Distribution Board/Parts and Parameters Master.xlsx
+++ b/astromech/Electrical/Power Distribution Board/Parts and Parameters Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\highf\Documents\GitHub\ue4\astromech\Electrical\Power Distribution Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08928747-765F-43AE-928A-F3835E5CA038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DFD1BE3-33B3-4DA4-8D22-FCFD39E306C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7289D41D-893F-4A0D-B079-C6690FDA4D7C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Part</t>
   </si>
@@ -57,6 +57,15 @@
   </si>
   <si>
     <t>KiCad Component</t>
+  </si>
+  <si>
+    <t>KiCad Footprint</t>
+  </si>
+  <si>
+    <t>Fuse:Fuseholder_Blade_Mini_Keystone_3568</t>
+  </si>
+  <si>
+    <t>Fuse</t>
   </si>
 </sst>
 </file>
@@ -411,16 +420,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66C6858F-B77B-4267-919C-E8D82019B723}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" customWidth="1"/>
     <col min="2" max="2" width="13.140625" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="5" width="18.85546875" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="41.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -433,8 +443,11 @@
       <c r="D1" t="s">
         <v>6</v>
       </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -443,6 +456,12 @@
       </c>
       <c r="C2" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>